<commit_message>
Add and expand Russian design specs and assets
Add multiple primary design specifications (movement, typing, dodge/initiative mechanics) in Russian and a terminology file; include supporting PNG and XLSX assets. Update existing design docs: fix typos and wording in Pokemon RE Concept (e.g., 'регулярный'), adjust initiative/OD/reaction rules, clarify passive/active dodge behavior and multi-target test resolution. Remove obsolete .txt artifacts and rename some spec files for consistency. Several binary design files (.docx, .xlsx) were also updated.

These changes expand and clarify core tactical and strategic rules for the project.
</commit_message>
<xml_diff>
--- a/design/Pokemon RE Standard_states.xlsx
+++ b/design/Pokemon RE Standard_states.xlsx
@@ -7,15 +7,15 @@
     <workbookView xWindow="240" yWindow="60" windowWidth="20115" windowHeight="8010" activeTab="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Лист2" sheetId="2" r:id="rId1"/>
-    <sheet name="Лист3" sheetId="3" r:id="rId2"/>
+    <sheet name="Краткий" sheetId="2" r:id="rId1"/>
+    <sheet name="Полный" sheetId="3" r:id="rId2"/>
   </sheets>
   <calcPr calcId="145621"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="175">
   <si>
     <t>Среднее значение</t>
   </si>
@@ -489,13 +489,72 @@
   </si>
   <si>
     <t>(+30 макс.бонус)</t>
+  </si>
+  <si>
+    <t>Пассивный уворот 5+</t>
+  </si>
+  <si>
+    <t>Пассивный уворот 8+</t>
+  </si>
+  <si>
+    <t>Пассивный уворот 13+</t>
+  </si>
+  <si>
+    <t>Пассивный уворот 18+</t>
+  </si>
+  <si>
+    <t>Пассивный уворот 23+</t>
+  </si>
+  <si>
+    <t>Пассивный уворот 25+</t>
+  </si>
+  <si>
+    <t>Пассивный уворот 28+</t>
+  </si>
+  <si>
+    <t>Базовая Быстрота 1 клетка</t>
+  </si>
+  <si>
+    <t>Базовая Быстрота 2 клетки</t>
+  </si>
+  <si>
+    <t>Базовая Быстрота 3 клетки</t>
+  </si>
+  <si>
+    <t>Базовая Быстрота 4 клетки</t>
+  </si>
+  <si>
+    <t>Базовая Быстрота 5 клеток</t>
+  </si>
+  <si>
+    <t>Базовая Быстрота 6 клеток</t>
+  </si>
+  <si>
+    <t>Базовая Быстрота 7 клеток</t>
+  </si>
+  <si>
+    <t>Базовая Быстрота 8 клеток</t>
+  </si>
+  <si>
+    <t>Базовая Быстрота 9 клеток</t>
+  </si>
+  <si>
+    <t>Базовая Быстрота 10 клеток</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+      <scheme val="minor"/>
+    </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -505,12 +564,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="65"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="8">
@@ -599,10 +664,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -625,7 +691,22 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -634,20 +715,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="20% - Акцент1" xfId="1" builtinId="30"/>
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1007,7 +1083,7 @@
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A2" s="9">
+      <c r="A2" s="14">
         <v>1</v>
       </c>
       <c r="B2" s="1">
@@ -1016,12 +1092,12 @@
       <c r="C2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="L2" s="11" t="s">
+      <c r="L2" s="10" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A3" s="9"/>
+      <c r="A3" s="14"/>
       <c r="B3" s="1">
         <v>3</v>
       </c>
@@ -1031,7 +1107,7 @@
       <c r="L3" s="13"/>
     </row>
     <row r="4" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="10"/>
+      <c r="A4" s="15"/>
       <c r="B4" s="2">
         <v>5</v>
       </c>
@@ -1045,7 +1121,7 @@
       <c r="L4" s="13"/>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A5" s="9">
+      <c r="A5" s="14">
         <v>2</v>
       </c>
       <c r="B5" s="1">
@@ -1065,7 +1141,7 @@
       </c>
     </row>
     <row r="6" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="10"/>
+      <c r="A6" s="15"/>
       <c r="B6" s="2">
         <v>9</v>
       </c>
@@ -1081,10 +1157,10 @@
       <c r="G6" s="4"/>
       <c r="I6" s="4"/>
       <c r="K6" s="4"/>
-      <c r="L6" s="12"/>
+      <c r="L6" s="11"/>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A7" s="9">
+      <c r="A7" s="14">
         <v>3</v>
       </c>
       <c r="B7" s="1">
@@ -1099,12 +1175,12 @@
       <c r="E7" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="L7" s="11" t="s">
+      <c r="L7" s="10" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="8" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="10"/>
+      <c r="A8" s="15"/>
       <c r="B8" s="2">
         <v>13</v>
       </c>
@@ -1125,10 +1201,10 @@
       </c>
       <c r="I8" s="4"/>
       <c r="K8" s="4"/>
-      <c r="L8" s="12"/>
+      <c r="L8" s="11"/>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A9" s="9">
+      <c r="A9" s="14">
         <v>4</v>
       </c>
       <c r="B9" s="1">
@@ -1149,12 +1225,12 @@
       <c r="G9" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="L9" s="11" t="s">
+      <c r="L9" s="10" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="10" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="10"/>
+      <c r="A10" s="15"/>
       <c r="B10" s="2">
         <v>17</v>
       </c>
@@ -1175,10 +1251,10 @@
       </c>
       <c r="I10" s="4"/>
       <c r="K10" s="4"/>
-      <c r="L10" s="12"/>
+      <c r="L10" s="11"/>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A11" s="9">
+      <c r="A11" s="14">
         <v>5</v>
       </c>
       <c r="D11" s="1">
@@ -1199,12 +1275,12 @@
       <c r="I11" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="L11" s="11" t="s">
+      <c r="L11" s="10" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="12" spans="1:12" s="2" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="10"/>
+      <c r="A12" s="15"/>
       <c r="C12" s="4"/>
       <c r="D12" s="2">
         <v>21</v>
@@ -1225,10 +1301,10 @@
         <v>17</v>
       </c>
       <c r="K12" s="4"/>
-      <c r="L12" s="12"/>
+      <c r="L12" s="11"/>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A13" s="9">
+      <c r="A13" s="14">
         <v>6</v>
       </c>
       <c r="D13" s="1">
@@ -1249,12 +1325,12 @@
       <c r="I13" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="L13" s="11" t="s">
+      <c r="L13" s="10" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="14" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="10"/>
+      <c r="A14" s="15"/>
       <c r="C14" s="4"/>
       <c r="E14" s="4"/>
       <c r="F14" s="2">
@@ -1275,10 +1351,10 @@
       <c r="K14" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="L14" s="12"/>
+      <c r="L14" s="11"/>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A15" s="9">
+      <c r="A15" s="14">
         <v>7</v>
       </c>
       <c r="F15" s="1">
@@ -1299,12 +1375,12 @@
       <c r="K15" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="L15" s="11" t="s">
+      <c r="L15" s="10" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="16" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="10"/>
+      <c r="A16" s="15"/>
       <c r="C16" s="4"/>
       <c r="E16" s="4"/>
       <c r="F16" s="2">
@@ -1325,10 +1401,10 @@
       <c r="K16" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="L16" s="12"/>
+      <c r="L16" s="11"/>
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A17" s="9">
+      <c r="A17" s="14">
         <v>8</v>
       </c>
       <c r="H17" s="1">
@@ -1343,12 +1419,12 @@
       <c r="K17" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="L17" s="11" t="s">
+      <c r="L17" s="10" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="18" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="10"/>
+      <c r="A18" s="15"/>
       <c r="C18" s="4"/>
       <c r="E18" s="4"/>
       <c r="G18" s="4"/>
@@ -1364,10 +1440,10 @@
       <c r="K18" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="L18" s="12"/>
+      <c r="L18" s="11"/>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A19" s="9">
+      <c r="A19" s="14">
         <v>9</v>
       </c>
       <c r="H19" s="1">
@@ -1382,12 +1458,12 @@
       <c r="K19" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="L19" s="11" t="s">
+      <c r="L19" s="10" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="20" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="10"/>
+      <c r="A20" s="15"/>
       <c r="C20" s="4"/>
       <c r="E20" s="4"/>
       <c r="G20" s="4"/>
@@ -1398,10 +1474,10 @@
       <c r="K20" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="L20" s="12"/>
+      <c r="L20" s="11"/>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A21" s="9">
+      <c r="A21" s="14">
         <v>10</v>
       </c>
       <c r="J21" s="1">
@@ -1410,12 +1486,12 @@
       <c r="K21" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="L21" s="11" t="s">
+      <c r="L21" s="10" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="22" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="10"/>
+      <c r="A22" s="15"/>
       <c r="C22" s="4"/>
       <c r="E22" s="4"/>
       <c r="G22" s="4"/>
@@ -1426,48 +1502,36 @@
       <c r="K22" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="L22" s="12"/>
+      <c r="L22" s="11"/>
     </row>
     <row r="23" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="B23" s="8">
+      <c r="B23" s="12">
         <v>1</v>
       </c>
-      <c r="C23" s="8"/>
-      <c r="D23" s="8">
+      <c r="C23" s="12"/>
+      <c r="D23" s="12">
         <v>2</v>
       </c>
-      <c r="E23" s="8"/>
-      <c r="F23" s="8">
+      <c r="E23" s="12"/>
+      <c r="F23" s="12">
         <v>2</v>
       </c>
-      <c r="G23" s="8"/>
-      <c r="H23" s="8">
+      <c r="G23" s="12"/>
+      <c r="H23" s="12">
         <v>3</v>
       </c>
-      <c r="I23" s="8"/>
-      <c r="J23" s="8">
+      <c r="I23" s="12"/>
+      <c r="J23" s="12">
         <v>3</v>
       </c>
-      <c r="K23" s="8"/>
+      <c r="K23" s="12"/>
       <c r="L23" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="25">
-    <mergeCell ref="L19:L20"/>
-    <mergeCell ref="L21:L22"/>
-    <mergeCell ref="H23:I23"/>
-    <mergeCell ref="J23:K23"/>
-    <mergeCell ref="L2:L4"/>
-    <mergeCell ref="L5:L6"/>
-    <mergeCell ref="L7:L8"/>
-    <mergeCell ref="L9:L10"/>
-    <mergeCell ref="L11:L12"/>
-    <mergeCell ref="L13:L14"/>
-    <mergeCell ref="L15:L16"/>
-    <mergeCell ref="L17:L18"/>
     <mergeCell ref="D23:E23"/>
     <mergeCell ref="F23:G23"/>
     <mergeCell ref="A2:A4"/>
@@ -1481,6 +1545,18 @@
     <mergeCell ref="A19:A20"/>
     <mergeCell ref="A21:A22"/>
     <mergeCell ref="B23:C23"/>
+    <mergeCell ref="L19:L20"/>
+    <mergeCell ref="L21:L22"/>
+    <mergeCell ref="H23:I23"/>
+    <mergeCell ref="J23:K23"/>
+    <mergeCell ref="L2:L4"/>
+    <mergeCell ref="L5:L6"/>
+    <mergeCell ref="L7:L8"/>
+    <mergeCell ref="L9:L10"/>
+    <mergeCell ref="L11:L12"/>
+    <mergeCell ref="L13:L14"/>
+    <mergeCell ref="L15:L16"/>
+    <mergeCell ref="L17:L18"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="89" orientation="landscape" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
@@ -1489,7 +1565,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:X61"/>
+  <dimension ref="A1:X63"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.7109375" style="6" customWidth="1"/>
@@ -1520,1028 +1596,1120 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="16" t="s">
         <v>152</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14" t="s">
+      <c r="B1" s="16"/>
+      <c r="C1" s="16" t="s">
         <v>153</v>
       </c>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14" t="s">
+      <c r="D1" s="16"/>
+      <c r="E1" s="16" t="s">
         <v>153</v>
       </c>
-      <c r="F1" s="14"/>
-      <c r="G1" s="14" t="s">
+      <c r="F1" s="16"/>
+      <c r="G1" s="16" t="s">
         <v>154</v>
       </c>
-      <c r="H1" s="14"/>
-      <c r="I1" s="14" t="s">
+      <c r="H1" s="16"/>
+      <c r="I1" s="16" t="s">
         <v>154</v>
       </c>
-      <c r="J1" s="14"/>
-      <c r="K1" s="14" t="s">
+      <c r="J1" s="16"/>
+      <c r="K1" s="16" t="s">
         <v>155</v>
       </c>
-      <c r="L1" s="14"/>
-      <c r="M1" s="14" t="s">
+      <c r="L1" s="16"/>
+      <c r="M1" s="16" t="s">
         <v>155</v>
       </c>
-      <c r="N1" s="14"/>
-      <c r="O1" s="14" t="s">
+      <c r="N1" s="16"/>
+      <c r="O1" s="16" t="s">
         <v>156</v>
       </c>
-      <c r="P1" s="14"/>
-      <c r="Q1" s="14" t="s">
+      <c r="P1" s="16"/>
+      <c r="Q1" s="16" t="s">
         <v>156</v>
       </c>
-      <c r="R1" s="14"/>
-      <c r="S1" s="14" t="s">
+      <c r="R1" s="16"/>
+      <c r="S1" s="16" t="s">
         <v>157</v>
       </c>
-      <c r="T1" s="14"/>
-      <c r="U1" s="14"/>
-      <c r="V1" s="14"/>
-      <c r="W1" s="14"/>
-      <c r="X1" s="14"/>
-    </row>
-    <row r="2" spans="1:24" ht="45" x14ac:dyDescent="0.25">
-      <c r="A2" s="6" t="s">
+      <c r="T1" s="16"/>
+      <c r="U1" s="16"/>
+      <c r="V1" s="16"/>
+      <c r="W1" s="16"/>
+      <c r="X1" s="16"/>
+    </row>
+    <row r="2" spans="1:24" s="8" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="16" t="s">
+        <v>165</v>
+      </c>
+      <c r="B2" s="16"/>
+      <c r="C2" s="16" t="s">
+        <v>166</v>
+      </c>
+      <c r="D2" s="16"/>
+      <c r="E2" s="16" t="s">
+        <v>167</v>
+      </c>
+      <c r="F2" s="16"/>
+      <c r="G2" s="16" t="s">
+        <v>168</v>
+      </c>
+      <c r="H2" s="16"/>
+      <c r="I2" s="16" t="s">
+        <v>169</v>
+      </c>
+      <c r="J2" s="16"/>
+      <c r="K2" s="16" t="s">
+        <v>170</v>
+      </c>
+      <c r="L2" s="16"/>
+      <c r="M2" s="16" t="s">
+        <v>171</v>
+      </c>
+      <c r="N2" s="16"/>
+      <c r="O2" s="16" t="s">
+        <v>172</v>
+      </c>
+      <c r="P2" s="16"/>
+      <c r="Q2" s="16" t="s">
+        <v>173</v>
+      </c>
+      <c r="R2" s="16"/>
+      <c r="S2" s="16" t="s">
+        <v>174</v>
+      </c>
+      <c r="T2" s="16"/>
+    </row>
+    <row r="3" spans="1:24" s="9" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="17" t="s">
+        <v>158</v>
+      </c>
+      <c r="B3" s="17"/>
+      <c r="C3" s="17" t="s">
+        <v>159</v>
+      </c>
+      <c r="D3" s="17"/>
+      <c r="E3" s="17" t="s">
+        <v>160</v>
+      </c>
+      <c r="F3" s="17"/>
+      <c r="G3" s="17" t="s">
+        <v>161</v>
+      </c>
+      <c r="H3" s="17"/>
+      <c r="I3" s="17" t="s">
+        <v>162</v>
+      </c>
+      <c r="J3" s="17"/>
+      <c r="K3" s="17" t="s">
+        <v>163</v>
+      </c>
+      <c r="L3" s="17"/>
+      <c r="M3" s="17"/>
+      <c r="N3" s="17"/>
+      <c r="O3" s="17"/>
+      <c r="P3" s="17"/>
+      <c r="Q3" s="17" t="s">
+        <v>164</v>
+      </c>
+      <c r="R3" s="17"/>
+      <c r="S3" s="17"/>
+      <c r="T3" s="17"/>
+    </row>
+    <row r="4" spans="1:24" ht="45" x14ac:dyDescent="0.25">
+      <c r="A4" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B4" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C4" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="7" t="s">
+      <c r="D4" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E4" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="F2" s="7" t="s">
+      <c r="F4" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="G2" s="6" t="s">
+      <c r="G4" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="H2" s="7" t="s">
+      <c r="H4" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="I2" s="6" t="s">
+      <c r="I4" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="J2" s="7" t="s">
+      <c r="J4" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="K2" s="6" t="s">
+      <c r="K4" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="L2" s="7" t="s">
+      <c r="L4" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="M2" s="6" t="s">
+      <c r="M4" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="N2" s="7" t="s">
+      <c r="N4" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="O2" s="6" t="s">
+      <c r="O4" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="P2" s="7" t="s">
+      <c r="P4" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="Q2" s="6" t="s">
+      <c r="Q4" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="R2" s="7" t="s">
+      <c r="R4" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="S2" s="6" t="s">
+      <c r="S4" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="T2" s="7" t="s">
+      <c r="T4" s="7" t="s">
         <v>43</v>
-      </c>
-    </row>
-    <row r="3" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A3" s="6">
-        <v>5.5</v>
-      </c>
-      <c r="B3" s="7" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="4" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A4" s="6">
-        <v>6.5</v>
-      </c>
-      <c r="B4" s="7" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="5" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A5" s="6">
-        <v>7.5</v>
+        <v>5.5</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A6" s="6">
-        <v>8.5</v>
+        <v>6.5</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="7" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A7" s="6">
-        <v>9.5</v>
+        <v>7.5</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A8" s="6">
-        <v>10.5</v>
+        <v>8.5</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="C8" s="6">
-        <v>11</v>
-      </c>
-      <c r="D8" s="7" t="s">
-        <v>8</v>
+        <v>60</v>
       </c>
     </row>
     <row r="9" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A9" s="6">
+        <v>9.5</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A10" s="6">
+        <v>10.5</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C10" s="6">
+        <v>11</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A11" s="6">
         <v>11.5</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B11" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="C9" s="6">
+      <c r="C11" s="6">
         <v>12</v>
       </c>
-      <c r="D9" s="7" t="s">
+      <c r="D11" s="7" t="s">
         <v>62</v>
-      </c>
-    </row>
-    <row r="10" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="B10" s="7">
-        <v>2</v>
-      </c>
-      <c r="C10" s="6">
-        <v>13</v>
-      </c>
-      <c r="D10" s="7" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="11" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="C11" s="6">
-        <v>14</v>
-      </c>
-      <c r="D11" s="7" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="12" spans="1:24" x14ac:dyDescent="0.25">
       <c r="C12" s="6">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="13" spans="1:24" x14ac:dyDescent="0.25">
       <c r="C13" s="6">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>64</v>
-      </c>
-      <c r="E13" s="6">
-        <v>16.5</v>
-      </c>
-      <c r="F13" s="7" t="s">
-        <v>13</v>
+        <v>63</v>
       </c>
     </row>
     <row r="14" spans="1:24" x14ac:dyDescent="0.25">
       <c r="C14" s="6">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="E14" s="6">
-        <v>17.5</v>
-      </c>
-      <c r="F14" s="7" t="s">
-        <v>68</v>
+        <v>10</v>
       </c>
     </row>
     <row r="15" spans="1:24" x14ac:dyDescent="0.25">
       <c r="C15" s="6">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E15" s="6">
-        <v>18.5</v>
+        <v>16.5</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="16" spans="1:24" x14ac:dyDescent="0.25">
       <c r="C16" s="6">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E16" s="6">
-        <v>19.5</v>
+        <v>17.5</v>
       </c>
       <c r="F16" s="7" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="17" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C17" s="6">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E17" s="6">
-        <v>20.5</v>
+        <v>18.5</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="18" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C18" s="6">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="E18" s="6">
-        <v>21.5</v>
+        <v>19.5</v>
       </c>
       <c r="F18" s="7" t="s">
-        <v>70</v>
-      </c>
-      <c r="G18" s="6">
-        <v>22</v>
-      </c>
-      <c r="H18" s="7" t="s">
-        <v>18</v>
+        <v>69</v>
       </c>
     </row>
     <row r="19" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C19" s="6">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E19" s="6">
-        <v>22.5</v>
+        <v>20.5</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="G19" s="6">
-        <v>23</v>
-      </c>
-      <c r="H19" s="7" t="s">
-        <v>74</v>
+        <v>15</v>
       </c>
     </row>
     <row r="20" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C20" s="6">
+        <v>21</v>
+      </c>
+      <c r="D20" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="E20" s="6">
+        <v>21.5</v>
+      </c>
+      <c r="F20" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="G20" s="6">
+        <v>22</v>
+      </c>
+      <c r="H20" s="7" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="21" spans="3:12" x14ac:dyDescent="0.25">
+      <c r="C21" s="6">
+        <v>22</v>
+      </c>
+      <c r="D21" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="E21" s="6">
+        <v>22.5</v>
+      </c>
+      <c r="F21" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="G21" s="6">
         <v>23</v>
       </c>
-      <c r="D20" s="7" t="s">
+      <c r="H21" s="7" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="22" spans="3:12" x14ac:dyDescent="0.25">
+      <c r="C22" s="6">
+        <v>23</v>
+      </c>
+      <c r="D22" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="E20" s="6">
+      <c r="E22" s="6">
         <v>23.5</v>
       </c>
-      <c r="F20" s="7" t="s">
+      <c r="F22" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="G20" s="6">
+      <c r="G22" s="6">
         <v>24</v>
       </c>
-      <c r="H20" s="7" t="s">
+      <c r="H22" s="7" t="s">
         <v>19</v>
-      </c>
-    </row>
-    <row r="21" spans="3:12" x14ac:dyDescent="0.25">
-      <c r="E21" s="6">
-        <v>24.5</v>
-      </c>
-      <c r="F21" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="G21" s="6">
-        <v>25</v>
-      </c>
-      <c r="H21" s="7" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="22" spans="3:12" x14ac:dyDescent="0.25">
-      <c r="E22" s="6">
-        <v>25.5</v>
-      </c>
-      <c r="F22" s="7" t="s">
-        <v>72</v>
-      </c>
-      <c r="G22" s="6">
-        <v>26</v>
-      </c>
-      <c r="H22" s="7" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="23" spans="3:12" x14ac:dyDescent="0.25">
       <c r="E23" s="6">
-        <v>26.5</v>
+        <v>24.5</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>41</v>
+        <v>32</v>
       </c>
       <c r="G23" s="6">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="H23" s="7" t="s">
-        <v>76</v>
-      </c>
-      <c r="I23" s="6">
-        <v>27.5</v>
-      </c>
-      <c r="J23" s="7" t="s">
-        <v>23</v>
+        <v>75</v>
       </c>
     </row>
     <row r="24" spans="3:12" x14ac:dyDescent="0.25">
       <c r="E24" s="6">
-        <v>27.5</v>
+        <v>25.5</v>
       </c>
       <c r="F24" s="7" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G24" s="6">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="H24" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="I24" s="6">
-        <v>28.5</v>
-      </c>
-      <c r="J24" s="7" t="s">
-        <v>80</v>
+        <v>20</v>
       </c>
     </row>
     <row r="25" spans="3:12" x14ac:dyDescent="0.25">
       <c r="E25" s="6">
+        <v>26.5</v>
+      </c>
+      <c r="F25" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="G25" s="6">
+        <v>27</v>
+      </c>
+      <c r="H25" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="I25" s="6">
+        <v>27.5</v>
+      </c>
+      <c r="J25" s="7" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="26" spans="3:12" x14ac:dyDescent="0.25">
+      <c r="E26" s="6">
+        <v>27.5</v>
+      </c>
+      <c r="F26" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="G26" s="6">
+        <v>28</v>
+      </c>
+      <c r="H26" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="I26" s="6">
         <v>28.5</v>
       </c>
-      <c r="F25" s="7" t="s">
+      <c r="J26" s="7" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="27" spans="3:12" x14ac:dyDescent="0.25">
+      <c r="E27" s="6">
+        <v>28.5</v>
+      </c>
+      <c r="F27" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="G25" s="6">
+      <c r="G27" s="6">
         <v>29</v>
       </c>
-      <c r="H25" s="7" t="s">
+      <c r="H27" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="I25" s="6">
+      <c r="I27" s="6">
         <v>29.5</v>
       </c>
-      <c r="J25" s="7" t="s">
+      <c r="J27" s="7" t="s">
         <v>24</v>
-      </c>
-    </row>
-    <row r="26" spans="3:12" x14ac:dyDescent="0.25">
-      <c r="G26" s="6">
-        <v>30</v>
-      </c>
-      <c r="H26" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="I26" s="6">
-        <v>30.5</v>
-      </c>
-      <c r="J26" s="7" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="27" spans="3:12" x14ac:dyDescent="0.25">
-      <c r="G27" s="6">
-        <v>31</v>
-      </c>
-      <c r="H27" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="I27" s="6">
-        <v>31.5</v>
-      </c>
-      <c r="J27" s="7" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="28" spans="3:12" x14ac:dyDescent="0.25">
       <c r="G28" s="6">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="H28" s="7" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="I28" s="6">
-        <v>32.5</v>
+        <v>30.5</v>
       </c>
       <c r="J28" s="7" t="s">
-        <v>82</v>
-      </c>
-      <c r="K28" s="6">
-        <v>33</v>
-      </c>
-      <c r="L28" s="7" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
     </row>
     <row r="29" spans="3:12" x14ac:dyDescent="0.25">
       <c r="G29" s="6">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="H29" s="7" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="I29" s="6">
-        <v>33.5</v>
+        <v>31.5</v>
       </c>
       <c r="J29" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="K29" s="6">
-        <v>34</v>
-      </c>
-      <c r="L29" s="7" t="s">
-        <v>87</v>
+        <v>25</v>
       </c>
     </row>
     <row r="30" spans="3:12" x14ac:dyDescent="0.25">
       <c r="G30" s="6">
+        <v>32</v>
+      </c>
+      <c r="H30" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="I30" s="6">
+        <v>32.5</v>
+      </c>
+      <c r="J30" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="K30" s="6">
+        <v>33</v>
+      </c>
+      <c r="L30" s="7" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="31" spans="3:12" x14ac:dyDescent="0.25">
+      <c r="G31" s="6">
+        <v>33</v>
+      </c>
+      <c r="H31" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="I31" s="6">
+        <v>33.5</v>
+      </c>
+      <c r="J31" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="K31" s="6">
         <v>34</v>
       </c>
-      <c r="H30" s="7" t="s">
+      <c r="L31" s="7" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="32" spans="3:12" x14ac:dyDescent="0.25">
+      <c r="G32" s="6">
+        <v>34</v>
+      </c>
+      <c r="H32" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="I30" s="6">
+      <c r="I32" s="6">
         <v>34.5</v>
       </c>
-      <c r="J30" s="7" t="s">
+      <c r="J32" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="K30" s="6">
+      <c r="K32" s="6">
         <v>35</v>
       </c>
-      <c r="L30" s="7" t="s">
+      <c r="L32" s="7" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="31" spans="3:12" x14ac:dyDescent="0.25">
-      <c r="I31" s="6">
+    <row r="33" spans="9:18" x14ac:dyDescent="0.25">
+      <c r="I33" s="6">
         <v>35.5</v>
       </c>
-      <c r="J31" s="7" t="s">
+      <c r="J33" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="K31" s="6">
+      <c r="K33" s="6">
         <v>36</v>
       </c>
-      <c r="L31" s="7" t="s">
+      <c r="L33" s="7" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="32" spans="3:12" x14ac:dyDescent="0.25">
-      <c r="I32" s="6">
+    <row r="34" spans="9:18" x14ac:dyDescent="0.25">
+      <c r="I34" s="6">
         <v>36.5</v>
       </c>
-      <c r="J32" s="7" t="s">
+      <c r="J34" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="K32" s="6">
+      <c r="K34" s="6">
         <v>37</v>
       </c>
-      <c r="L32" s="7" t="s">
+      <c r="L34" s="7" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="33" spans="9:20" x14ac:dyDescent="0.25">
-      <c r="I33" s="6">
+    <row r="35" spans="9:18" x14ac:dyDescent="0.25">
+      <c r="I35" s="6">
         <v>37.5</v>
       </c>
-      <c r="J33" s="7" t="s">
+      <c r="J35" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="K33" s="6">
+      <c r="K35" s="6">
         <v>38</v>
       </c>
-      <c r="L33" s="7" t="s">
+      <c r="L35" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="M33" s="6">
+      <c r="M35" s="6">
         <v>38.5</v>
       </c>
-      <c r="N33" s="7" t="s">
+      <c r="N35" s="7" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="34" spans="9:20" x14ac:dyDescent="0.25">
-      <c r="I34" s="6">
+    <row r="36" spans="9:18" x14ac:dyDescent="0.25">
+      <c r="I36" s="6">
         <v>38.5</v>
       </c>
-      <c r="J34" s="7" t="s">
+      <c r="J36" s="7" t="s">
         <v>85</v>
       </c>
-      <c r="K34" s="6">
+      <c r="K36" s="6">
         <v>39</v>
       </c>
-      <c r="L34" s="7" t="s">
+      <c r="L36" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="M34" s="6">
+      <c r="M36" s="6">
         <v>39.5</v>
       </c>
-      <c r="N34" s="7" t="s">
+      <c r="N36" s="7" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="35" spans="9:20" x14ac:dyDescent="0.25">
-      <c r="I35" s="6">
+    <row r="37" spans="9:18" x14ac:dyDescent="0.25">
+      <c r="I37" s="6">
         <v>39.5</v>
       </c>
-      <c r="J35" s="7" t="s">
+      <c r="J37" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="K35" s="6">
+      <c r="K37" s="6">
         <v>40</v>
       </c>
-      <c r="L35" s="7" t="s">
+      <c r="L37" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="M35" s="6">
+      <c r="M37" s="6">
         <v>40.5</v>
       </c>
-      <c r="N35" s="7" t="s">
+      <c r="N37" s="7" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="36" spans="9:20" x14ac:dyDescent="0.25">
-      <c r="I36" s="6" t="s">
+    <row r="38" spans="9:18" x14ac:dyDescent="0.25">
+      <c r="I38" s="6" t="s">
         <v>151</v>
       </c>
-      <c r="J36" s="7" t="s">
+      <c r="J38" s="7" t="s">
         <v>151</v>
       </c>
-      <c r="K36" s="6">
+      <c r="K38" s="6">
         <v>41</v>
       </c>
-      <c r="L36" s="7" t="s">
+      <c r="L38" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="M36" s="6">
+      <c r="M38" s="6">
         <v>41.5</v>
       </c>
-      <c r="N36" s="7" t="s">
+      <c r="N38" s="7" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="37" spans="9:20" x14ac:dyDescent="0.25">
-      <c r="K37" s="6">
+    <row r="39" spans="9:18" x14ac:dyDescent="0.25">
+      <c r="K39" s="6">
         <v>42</v>
       </c>
-      <c r="L37" s="7" t="s">
+      <c r="L39" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="M37" s="6">
+      <c r="M39" s="6">
         <v>42.5</v>
       </c>
-      <c r="N37" s="7" t="s">
+      <c r="N39" s="7" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="38" spans="9:20" x14ac:dyDescent="0.25">
-      <c r="K38" s="6">
+    <row r="40" spans="9:18" x14ac:dyDescent="0.25">
+      <c r="K40" s="6">
         <v>43</v>
       </c>
-      <c r="L38" s="7" t="s">
+      <c r="L40" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="M38" s="6">
+      <c r="M40" s="6">
         <v>43.5</v>
       </c>
-      <c r="N38" s="7" t="s">
+      <c r="N40" s="7" t="s">
         <v>104</v>
       </c>
-      <c r="O38" s="6">
+      <c r="O40" s="6">
         <v>44</v>
       </c>
-      <c r="P38" s="7" t="s">
+      <c r="P40" s="7" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="39" spans="9:20" x14ac:dyDescent="0.25">
-      <c r="K39" s="6">
+    <row r="41" spans="9:18" x14ac:dyDescent="0.25">
+      <c r="K41" s="6">
         <v>44</v>
       </c>
-      <c r="L39" s="7" t="s">
+      <c r="L41" s="7" t="s">
         <v>97</v>
       </c>
-      <c r="M39" s="6">
+      <c r="M41" s="6">
         <v>44.5</v>
       </c>
-      <c r="N39" s="7" t="s">
+      <c r="N41" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="O39" s="6">
+      <c r="O41" s="6">
         <v>45</v>
       </c>
-      <c r="P39" s="7" t="s">
+      <c r="P41" s="7" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="40" spans="9:20" x14ac:dyDescent="0.25">
-      <c r="K40" s="6">
+    <row r="42" spans="9:18" x14ac:dyDescent="0.25">
+      <c r="K42" s="6">
         <v>45</v>
       </c>
-      <c r="L40" s="7" t="s">
+      <c r="L42" s="7" t="s">
         <v>98</v>
       </c>
-      <c r="M40" s="6">
+      <c r="M42" s="6">
         <v>45.5</v>
       </c>
-      <c r="N40" s="7" t="s">
+      <c r="N42" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="O40" s="6">
+      <c r="O42" s="6">
         <v>46</v>
       </c>
-      <c r="P40" s="7" t="s">
+      <c r="P42" s="7" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="41" spans="9:20" x14ac:dyDescent="0.25">
-      <c r="K41" s="6" t="s">
+    <row r="43" spans="9:18" x14ac:dyDescent="0.25">
+      <c r="K43" s="6" t="s">
         <v>151</v>
       </c>
-      <c r="L41" s="7" t="s">
+      <c r="L43" s="7" t="s">
         <v>151</v>
       </c>
-      <c r="M41" s="6">
+      <c r="M43" s="6">
         <v>46.5</v>
       </c>
-      <c r="N41" s="7" t="s">
+      <c r="N43" s="7" t="s">
         <v>107</v>
       </c>
-      <c r="O41" s="6">
+      <c r="O43" s="6">
         <v>47</v>
       </c>
-      <c r="P41" s="7" t="s">
+      <c r="P43" s="7" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="42" spans="9:20" x14ac:dyDescent="0.25">
-      <c r="M42" s="6">
+    <row r="44" spans="9:18" x14ac:dyDescent="0.25">
+      <c r="M44" s="6">
         <v>47.5</v>
       </c>
-      <c r="N42" s="7" t="s">
+      <c r="N44" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="O42" s="6">
+      <c r="O44" s="6">
         <v>48</v>
       </c>
-      <c r="P42" s="7" t="s">
+      <c r="P44" s="7" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="43" spans="9:20" x14ac:dyDescent="0.25">
-      <c r="M43" s="6">
+    <row r="45" spans="9:18" x14ac:dyDescent="0.25">
+      <c r="M45" s="6">
         <v>48.5</v>
       </c>
-      <c r="N43" s="7" t="s">
+      <c r="N45" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="O43" s="6">
+      <c r="O45" s="6">
         <v>49</v>
       </c>
-      <c r="P43" s="7" t="s">
+      <c r="P45" s="7" t="s">
         <v>117</v>
       </c>
-      <c r="Q43" s="6">
+      <c r="Q45" s="6">
         <v>50.5</v>
       </c>
-      <c r="R43" s="7" t="s">
+      <c r="R45" s="7" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="44" spans="9:20" x14ac:dyDescent="0.25">
-      <c r="M44" s="6">
+    <row r="46" spans="9:18" x14ac:dyDescent="0.25">
+      <c r="M46" s="6">
         <v>49.5</v>
       </c>
-      <c r="N44" s="7" t="s">
+      <c r="N46" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="O44" s="6">
+      <c r="O46" s="6">
         <v>50</v>
       </c>
-      <c r="P44" s="7" t="s">
+      <c r="P46" s="7" t="s">
         <v>118</v>
       </c>
-      <c r="Q44" s="6">
+      <c r="Q46" s="6">
         <v>51.5</v>
       </c>
-      <c r="R44" s="7" t="s">
+      <c r="R46" s="7" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="45" spans="9:20" x14ac:dyDescent="0.25">
-      <c r="M45" s="6">
+    <row r="47" spans="9:18" x14ac:dyDescent="0.25">
+      <c r="M47" s="6">
         <v>50.5</v>
       </c>
-      <c r="N45" s="7" t="s">
+      <c r="N47" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="O45" s="6">
+      <c r="O47" s="6">
         <v>51</v>
       </c>
-      <c r="P45" s="7" t="s">
+      <c r="P47" s="7" t="s">
         <v>119</v>
       </c>
-      <c r="Q45" s="6">
+      <c r="Q47" s="6">
         <v>52.5</v>
       </c>
-      <c r="R45" s="7" t="s">
+      <c r="R47" s="7" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="46" spans="9:20" x14ac:dyDescent="0.25">
-      <c r="M46" s="6" t="s">
+    <row r="48" spans="9:18" x14ac:dyDescent="0.25">
+      <c r="M48" s="6" t="s">
         <v>151</v>
       </c>
-      <c r="N46" s="7" t="s">
+      <c r="N48" s="7" t="s">
         <v>151</v>
       </c>
-      <c r="O46" s="6">
+      <c r="O48" s="6">
         <v>52</v>
       </c>
-      <c r="P46" s="7" t="s">
+      <c r="P48" s="7" t="s">
         <v>120</v>
       </c>
-      <c r="Q46" s="6">
+      <c r="Q48" s="6">
         <v>53.5</v>
       </c>
-      <c r="R46" s="7" t="s">
+      <c r="R48" s="7" t="s">
         <v>128</v>
-      </c>
-    </row>
-    <row r="47" spans="9:20" x14ac:dyDescent="0.25">
-      <c r="O47" s="6">
-        <v>53</v>
-      </c>
-      <c r="P47" s="7" t="s">
-        <v>121</v>
-      </c>
-      <c r="Q47" s="6">
-        <v>54.5</v>
-      </c>
-      <c r="R47" s="7" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="48" spans="9:20" x14ac:dyDescent="0.25">
-      <c r="O48" s="6">
-        <v>54</v>
-      </c>
-      <c r="P48" s="7" t="s">
-        <v>122</v>
-      </c>
-      <c r="Q48" s="6">
-        <v>55.5</v>
-      </c>
-      <c r="R48" s="7" t="s">
-        <v>130</v>
-      </c>
-      <c r="S48" s="6">
-        <v>55</v>
-      </c>
-      <c r="T48" s="7" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="49" spans="15:20" x14ac:dyDescent="0.25">
       <c r="O49" s="6">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="P49" s="7" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="Q49" s="6">
-        <v>56.5</v>
+        <v>54.5</v>
       </c>
       <c r="R49" s="7" t="s">
-        <v>131</v>
-      </c>
-      <c r="S49" s="6">
-        <v>56</v>
-      </c>
-      <c r="T49" s="7" t="s">
-        <v>139</v>
+        <v>129</v>
       </c>
     </row>
     <row r="50" spans="15:20" x14ac:dyDescent="0.25">
       <c r="O50" s="6">
+        <v>54</v>
+      </c>
+      <c r="P50" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="Q50" s="6">
+        <v>55.5</v>
+      </c>
+      <c r="R50" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="S50" s="6">
+        <v>55</v>
+      </c>
+      <c r="T50" s="7" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="51" spans="15:20" x14ac:dyDescent="0.25">
+      <c r="O51" s="6">
+        <v>55</v>
+      </c>
+      <c r="P51" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="Q51" s="6">
+        <v>56.5</v>
+      </c>
+      <c r="R51" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="S51" s="6">
         <v>56</v>
       </c>
-      <c r="P50" s="7" t="s">
+      <c r="T51" s="7" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="52" spans="15:20" x14ac:dyDescent="0.25">
+      <c r="O52" s="6">
+        <v>56</v>
+      </c>
+      <c r="P52" s="7" t="s">
         <v>124</v>
       </c>
-      <c r="Q50" s="6">
+      <c r="Q52" s="6">
         <v>57.5</v>
       </c>
-      <c r="R50" s="7" t="s">
+      <c r="R52" s="7" t="s">
         <v>132</v>
       </c>
-      <c r="S50" s="6">
+      <c r="S52" s="6">
         <v>57</v>
       </c>
-      <c r="T50" s="7" t="s">
+      <c r="T52" s="7" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="51" spans="15:20" x14ac:dyDescent="0.25">
-      <c r="O51" s="6" t="s">
+    <row r="53" spans="15:20" x14ac:dyDescent="0.25">
+      <c r="O53" s="6" t="s">
         <v>151</v>
       </c>
-      <c r="P51" s="7" t="s">
+      <c r="P53" s="7" t="s">
         <v>151</v>
       </c>
-      <c r="Q51" s="6">
+      <c r="Q53" s="6">
         <v>58.5</v>
       </c>
-      <c r="R51" s="7" t="s">
+      <c r="R53" s="7" t="s">
         <v>133</v>
       </c>
-      <c r="S51" s="6">
+      <c r="S53" s="6">
         <v>58</v>
       </c>
-      <c r="T51" s="7" t="s">
+      <c r="T53" s="7" t="s">
         <v>141</v>
-      </c>
-    </row>
-    <row r="52" spans="15:20" x14ac:dyDescent="0.25">
-      <c r="Q52" s="6">
-        <v>59.5</v>
-      </c>
-      <c r="R52" s="7" t="s">
-        <v>134</v>
-      </c>
-      <c r="S52" s="6">
-        <v>59</v>
-      </c>
-      <c r="T52" s="7" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="53" spans="15:20" x14ac:dyDescent="0.25">
-      <c r="Q53" s="6">
-        <v>60.5</v>
-      </c>
-      <c r="R53" s="7" t="s">
-        <v>135</v>
-      </c>
-      <c r="S53" s="6">
-        <v>60</v>
-      </c>
-      <c r="T53" s="7" t="s">
-        <v>143</v>
       </c>
     </row>
     <row r="54" spans="15:20" x14ac:dyDescent="0.25">
       <c r="Q54" s="6">
-        <v>61.5</v>
+        <v>59.5</v>
       </c>
       <c r="R54" s="7" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="S54" s="6">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="T54" s="7" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
     </row>
     <row r="55" spans="15:20" x14ac:dyDescent="0.25">
       <c r="Q55" s="6">
+        <v>60.5</v>
+      </c>
+      <c r="R55" s="7" t="s">
+        <v>135</v>
+      </c>
+      <c r="S55" s="6">
+        <v>60</v>
+      </c>
+      <c r="T55" s="7" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="56" spans="15:20" x14ac:dyDescent="0.25">
+      <c r="Q56" s="6">
+        <v>61.5</v>
+      </c>
+      <c r="R56" s="7" t="s">
+        <v>136</v>
+      </c>
+      <c r="S56" s="6">
+        <v>61</v>
+      </c>
+      <c r="T56" s="7" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="57" spans="15:20" x14ac:dyDescent="0.25">
+      <c r="Q57" s="6">
         <v>62.5</v>
       </c>
-      <c r="R55" s="7" t="s">
+      <c r="R57" s="7" t="s">
         <v>137</v>
       </c>
-      <c r="S55" s="6">
+      <c r="S57" s="6">
         <v>62</v>
       </c>
-      <c r="T55" s="7" t="s">
+      <c r="T57" s="7" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="56" spans="15:20" x14ac:dyDescent="0.25">
-      <c r="Q56" s="6" t="s">
+    <row r="58" spans="15:20" x14ac:dyDescent="0.25">
+      <c r="Q58" s="6" t="s">
         <v>151</v>
       </c>
-      <c r="R56" s="7" t="s">
+      <c r="R58" s="7" t="s">
         <v>151</v>
       </c>
-      <c r="S56" s="6">
+      <c r="S58" s="6">
         <v>63</v>
       </c>
-      <c r="T56" s="7" t="s">
+      <c r="T58" s="7" t="s">
         <v>146</v>
-      </c>
-    </row>
-    <row r="57" spans="15:20" x14ac:dyDescent="0.25">
-      <c r="S57" s="6">
-        <v>64</v>
-      </c>
-      <c r="T57" s="7" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="58" spans="15:20" x14ac:dyDescent="0.25">
-      <c r="S58" s="6">
-        <v>65</v>
-      </c>
-      <c r="T58" s="7" t="s">
-        <v>148</v>
       </c>
     </row>
     <row r="59" spans="15:20" x14ac:dyDescent="0.25">
       <c r="S59" s="6">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="T59" s="7" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
     </row>
     <row r="60" spans="15:20" x14ac:dyDescent="0.25">
       <c r="S60" s="6">
+        <v>65</v>
+      </c>
+      <c r="T60" s="7" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="61" spans="15:20" x14ac:dyDescent="0.25">
+      <c r="S61" s="6">
+        <v>66</v>
+      </c>
+      <c r="T61" s="7" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="62" spans="15:20" x14ac:dyDescent="0.25">
+      <c r="S62" s="6">
         <v>67</v>
       </c>
-      <c r="T60" s="7" t="s">
+      <c r="T62" s="7" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="61" spans="15:20" x14ac:dyDescent="0.25">
-      <c r="S61" s="6" t="s">
+    <row r="63" spans="15:20" x14ac:dyDescent="0.25">
+      <c r="S63" s="6" t="s">
         <v>151</v>
       </c>
-      <c r="T61" s="7" t="s">
+      <c r="T63" s="7" t="s">
         <v>151</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="29">
+    <mergeCell ref="K3:P3"/>
+    <mergeCell ref="Q3:T3"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="E3:F3"/>
+    <mergeCell ref="G3:H3"/>
+    <mergeCell ref="I3:J3"/>
+    <mergeCell ref="W1:X1"/>
+    <mergeCell ref="Q1:R1"/>
+    <mergeCell ref="S1:T1"/>
+    <mergeCell ref="U1:V1"/>
+    <mergeCell ref="M1:N1"/>
+    <mergeCell ref="O1:P1"/>
     <mergeCell ref="K1:L1"/>
     <mergeCell ref="C1:D1"/>
     <mergeCell ref="E1:F1"/>
     <mergeCell ref="G1:H1"/>
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="I1:J1"/>
-    <mergeCell ref="W1:X1"/>
-    <mergeCell ref="Q1:R1"/>
-    <mergeCell ref="S1:T1"/>
-    <mergeCell ref="U1:V1"/>
-    <mergeCell ref="M1:N1"/>
-    <mergeCell ref="O1:P1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="G2:H2"/>
+    <mergeCell ref="I2:J2"/>
+    <mergeCell ref="K2:L2"/>
+    <mergeCell ref="M2:N2"/>
+    <mergeCell ref="O2:P2"/>
+    <mergeCell ref="Q2:R2"/>
+    <mergeCell ref="S2:T2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>

</xml_diff>